<commit_message>
Tarifa LP como tarifa de Nacional; razones sociales de Fletes empatadas por correo o a mano
- La tarifa sugerida es la «TARIFA LP» de Fletes (la «TARIFA» queda como referencia).
- La razón social de Fletes se empata con su transportista por nombre (sin prefijos ni S.A. de C.V.),
  por correo, o a mano con «Unir con…»; lo unido se recuerda al volver a importar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013L2S8grapiu9RE7gAXriRp
</commit_message>
<xml_diff>
--- a/tests/fletes-ejemplo.xlsx
+++ b/tests/fletes-ejemplo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:N12"/>
+  <dimension ref="B3:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -551,6 +551,35 @@
         <v>60</v>
       </c>
       <c r="N12" t="n">
+        <v>1.12</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LEON</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>300</v>
+      </c>
+      <c r="D13" t="n">
+        <v>260</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>MARIA PERSONA FISICA</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>45</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>trafico@fletes.example</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
         <v>1.12</v>
       </c>
     </row>

</xml_diff>